<commit_message>
chore: update coding-agents leaderboard (2026-08-30)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -609,7 +609,7 @@
         <v>0.642976619611059</v>
       </c>
       <c r="P2" t="n">
-        <v>1016.984589363497</v>
+        <v>994.513944278713</v>
       </c>
       <c r="Q2" t="n">
         <v>55738.30836457358</v>
@@ -627,16 +627,16 @@
         <v>14.40194046721888</v>
       </c>
       <c r="V2" t="n">
-        <v>3.720011838916402</v>
+        <v>3.804064019606651</v>
       </c>
       <c r="W2" t="n">
-        <v>0.06200019731527338</v>
+        <v>0.06340106699344419</v>
       </c>
       <c r="X2" t="n">
         <v>0.06943508774224974</v>
       </c>
       <c r="Y2" t="n">
-        <v>54.8074267275364</v>
+        <v>56.0457786290756</v>
       </c>
       <c r="Z2" t="n">
         <v>1.131237151919106</v>
@@ -703,7 +703,7 @@
         <v>1.368245231958763</v>
       </c>
       <c r="P3" t="n">
-        <v>638.1828345155545</v>
+        <v>724.694563327613</v>
       </c>
       <c r="Q3" t="n">
         <v>45251.51726804124</v>
@@ -721,16 +721,16 @@
         <v>11.08314725485995</v>
       </c>
       <c r="V3" t="n">
-        <v>5.83588202420383</v>
+        <v>5.139213015485393</v>
       </c>
       <c r="W3" t="n">
-        <v>0.09726470040339716</v>
+        <v>0.08565355025808988</v>
       </c>
       <c r="X3" t="n">
         <v>0.09022707873537468</v>
       </c>
       <c r="Y3" t="n">
-        <v>70.9068229677342</v>
+        <v>62.4421922806455</v>
       </c>
       <c r="Z3" t="n">
         <v>1.371725545335136</v>
@@ -785,10 +785,10 @@
         <v>57.7836323024055</v>
       </c>
       <c r="L4" t="n">
-        <v>2.168492783333491</v>
+        <v>2.030547294444435</v>
       </c>
       <c r="M4" t="n">
-        <v>1.676910955779601</v>
+        <v>1.538965466890545</v>
       </c>
       <c r="N4" t="n">
         <v>0.4915818275538894</v>
@@ -797,7 +797,7 @@
         <v>0.2407592811621368</v>
       </c>
       <c r="P4" t="n">
-        <v>343.367610073</v>
+        <v>325.9640798990283</v>
       </c>
       <c r="Q4" t="n">
         <v>24579.09137769447</v>
@@ -809,22 +809,22 @@
         <v>12037.96405810684</v>
       </c>
       <c r="T4" t="n">
-        <v>785.2494536795145</v>
+        <v>739.5647333206439</v>
       </c>
       <c r="U4" t="n">
-        <v>28.09779705111887</v>
+        <v>30.00662446997617</v>
       </c>
       <c r="V4" t="n">
-        <v>10.64687553726455</v>
+        <v>11.21532228062567</v>
       </c>
       <c r="W4" t="n">
-        <v>0.1774479256210759</v>
+        <v>0.1869220380104278</v>
       </c>
       <c r="X4" t="n">
-        <v>0.03558997875102737</v>
+        <v>0.03332597443609737</v>
       </c>
       <c r="Y4" t="n">
-        <v>71.5824400923225</v>
+        <v>75.40429419495599</v>
       </c>
       <c r="Z4" t="n">
         <v>2.478930941613821</v>
@@ -891,7 +891,7 @@
         <v>0.07637769011246485</v>
       </c>
       <c r="P5" t="n">
-        <v>613.755746714795</v>
+        <v>548.8307863739595</v>
       </c>
       <c r="Q5" t="n">
         <v>32127.57155576383</v>
@@ -909,16 +909,16 @@
         <v>27.72109542352386</v>
       </c>
       <c r="V5" t="n">
-        <v>5.955754039672741</v>
+        <v>6.660301059311051</v>
       </c>
       <c r="W5" t="n">
-        <v>0.09926256732787901</v>
+        <v>0.1110050176551842</v>
       </c>
       <c r="X5" t="n">
         <v>0.03607361053818275</v>
       </c>
       <c r="Y5" t="n">
-        <v>52.3458586379528</v>
+        <v>58.5382095053846</v>
       </c>
       <c r="Z5" t="n">
         <v>1.896283104541718</v>
@@ -985,7 +985,7 @@
         <v>0.2987502065370197</v>
       </c>
       <c r="P6" t="n">
-        <v>917.6825022622578</v>
+        <v>895.3932251241574</v>
       </c>
       <c r="Q6" t="n">
         <v>34600.18969072165</v>
@@ -1003,16 +1003,16 @@
         <v>36.43986803085358</v>
       </c>
       <c r="V6" t="n">
-        <v>3.903275936094821</v>
+        <v>4.000441289422161</v>
       </c>
       <c r="W6" t="n">
-        <v>0.06505459893491368</v>
+        <v>0.06667402149036936</v>
       </c>
       <c r="X6" t="n">
         <v>0.0274424704050328</v>
       </c>
       <c r="Y6" t="n">
-        <v>37.703878634959</v>
+        <v>38.6424519639669</v>
       </c>
       <c r="Z6" t="n">
         <v>1.725408665903012</v>
@@ -1058,7 +1058,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
         <v>59.5134408119521</v>
@@ -1079,7 +1079,7 @@
         <v>0.1156618241237113</v>
       </c>
       <c r="P7" t="n">
-        <v>595.4533867575117</v>
+        <v>771.6276580902694</v>
       </c>
       <c r="Q7" t="n">
         <v>51504.77661668229</v>
@@ -1097,16 +1097,16 @@
         <v>45.23673173150109</v>
       </c>
       <c r="V7" t="n">
-        <v>5.996785857851333</v>
+        <v>4.627628897536734</v>
       </c>
       <c r="W7" t="n">
-        <v>0.09994643096418888</v>
+        <v>0.07712714829227892</v>
       </c>
       <c r="X7" t="n">
         <v>0.0221059294454652</v>
       </c>
       <c r="Y7" t="n">
-        <v>86.49673973163031</v>
+        <v>66.74822510140891</v>
       </c>
       <c r="Z7" t="n">
         <v>1.155493620618399</v>
@@ -1173,7 +1173,7 @@
         <v>0.1498817592314902</v>
       </c>
       <c r="P8" t="n">
-        <v>2156.429177344399</v>
+        <v>1696.722364977395</v>
       </c>
       <c r="Q8" t="n">
         <v>48290.57678069354</v>
@@ -1191,16 +1191,16 @@
         <v>34.92400170745936</v>
       </c>
       <c r="V8" t="n">
-        <v>1.605552130346555</v>
+        <v>2.040557448344175</v>
       </c>
       <c r="W8" t="n">
-        <v>0.02675920217244258</v>
+        <v>0.03400929080573625</v>
       </c>
       <c r="X8" t="n">
         <v>0.02863360299820429</v>
       </c>
       <c r="Y8" t="n">
-        <v>22.3937689621518</v>
+        <v>28.4610952136161</v>
       </c>
       <c r="Z8" t="n">
         <v>1.194939637792499</v>
@@ -1267,7 +1267,7 @@
         <v>0.02030826248828491</v>
       </c>
       <c r="P9" t="n">
-        <v>1411.396240847372</v>
+        <v>1402.906852827542</v>
       </c>
       <c r="Q9" t="n">
         <v>68754.14777413307</v>
@@ -1285,16 +1285,16 @@
         <v>329.8695828083637</v>
       </c>
       <c r="V9" t="n">
-        <v>2.442653543329619</v>
+        <v>2.457434734030587</v>
       </c>
       <c r="W9" t="n">
-        <v>0.04071089238882698</v>
+        <v>0.04095724556717645</v>
       </c>
       <c r="X9" t="n">
         <v>0.003031501090480796</v>
       </c>
       <c r="Y9" t="n">
-        <v>48.71356872316349</v>
+        <v>49.0083483700717</v>
       </c>
       <c r="Z9" t="n">
         <v>0.8357197687606245</v>
@@ -1447,7 +1447,7 @@
         <v>0.1725414728209934</v>
       </c>
       <c r="P11" t="n">
-        <v>233.3760072292079</v>
+        <v>232.7940171020261</v>
       </c>
       <c r="Q11" t="n">
         <v>25497.47776476101</v>
@@ -1465,16 +1465,16 @@
         <v>60.63731862932376</v>
       </c>
       <c r="V11" t="n">
-        <v>14.54534292382237</v>
+        <v>14.58170659881505</v>
       </c>
       <c r="W11" t="n">
-        <v>0.2424223820637063</v>
+        <v>0.2430284433135842</v>
       </c>
       <c r="X11" t="n">
         <v>0.01649149438999777</v>
       </c>
       <c r="Y11" t="n">
-        <v>109.254923278034</v>
+        <v>109.528062972453</v>
       </c>
       <c r="Z11" t="n">
         <v>2.218869180355243</v>
@@ -1541,7 +1541,7 @@
         <v>0.07868562089971884</v>
       </c>
       <c r="P12" t="n">
-        <v>206.3949876563918</v>
+        <v>211.7154654996418</v>
       </c>
       <c r="Q12" t="n">
         <v>69809.11455014057</v>
@@ -1559,16 +1559,16 @@
         <v>68.63589797525123</v>
       </c>
       <c r="V12" t="n">
-        <v>16.28822057558375</v>
+        <v>15.87889234595326</v>
       </c>
       <c r="W12" t="n">
-        <v>0.2714703429263958</v>
+        <v>0.2646482057658877</v>
       </c>
       <c r="X12" t="n">
         <v>0.01456963527104403</v>
       </c>
       <c r="Y12" t="n">
-        <v>338.2306680158309</v>
+        <v>329.730822381791</v>
       </c>
       <c r="Z12" t="n">
         <v>0.8026189479473506</v>
@@ -1635,7 +1635,7 @@
         <v>0.1067159869793814</v>
       </c>
       <c r="P13" t="n">
-        <v>619.4867739280457</v>
+        <v>579.8133947356218</v>
       </c>
       <c r="Q13" t="n">
         <v>41492.56419868791</v>
@@ -1653,16 +1653,16 @@
         <v>136.2575680208481</v>
       </c>
       <c r="V13" t="n">
-        <v>5.152428155241987</v>
+        <v>5.504979920724816</v>
       </c>
       <c r="W13" t="n">
-        <v>0.08587380258736643</v>
+        <v>0.09174966534541361</v>
       </c>
       <c r="X13" t="n">
         <v>0.007339041893416113</v>
       </c>
       <c r="Y13" t="n">
-        <v>66.97893473268459</v>
+        <v>71.56192763985268</v>
       </c>
       <c r="Z13" t="n">
         <v>1.282101647780634</v>
@@ -1729,7 +1729,7 @@
         <v>0.01364774963448922</v>
       </c>
       <c r="P14" t="n">
-        <v>166.7517698995541</v>
+        <v>168.7844638728316</v>
       </c>
       <c r="Q14" t="n">
         <v>21435.03259137769</v>
@@ -1747,16 +1747,16 @@
         <v>654.5952122685204</v>
       </c>
       <c r="V14" t="n">
-        <v>18.82489744448763</v>
+        <v>18.59818667558767</v>
       </c>
       <c r="W14" t="n">
-        <v>0.3137482907414604</v>
+        <v>0.3099697779264611</v>
       </c>
       <c r="X14" t="n">
         <v>0.001527661646858779</v>
       </c>
       <c r="Y14" t="n">
-        <v>128.544558203427</v>
+        <v>126.996478820039</v>
       </c>
       <c r="Z14" t="n">
         <v>2.440774585299371</v>
@@ -1823,7 +1823,7 @@
         <v>0.110931870267104</v>
       </c>
       <c r="P15" t="n">
-        <v>1065.860868336992</v>
+        <v>1191.813234926616</v>
       </c>
       <c r="Q15" t="n">
         <v>55161.14899250234</v>
@@ -1841,16 +1841,16 @@
         <v>85.55045512028488</v>
       </c>
       <c r="V15" t="n">
-        <v>2.928599530868904</v>
+        <v>2.619101338621597</v>
       </c>
       <c r="W15" t="n">
-        <v>0.0488099921811484</v>
+        <v>0.04365168897702661</v>
       </c>
       <c r="X15" t="n">
         <v>0.01168900853413333</v>
       </c>
       <c r="Y15" t="n">
-        <v>51.7526730093464</v>
+        <v>46.2833834832341</v>
       </c>
       <c r="Z15" t="n">
         <v>0.9431395393303345</v>
@@ -1910,13 +1910,13 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="n">
-        <v>27463.54803186504</v>
+        <v>27938.56621368323</v>
       </c>
       <c r="R16" t="n">
-        <v>10833.09995313964</v>
+        <v>10985.54086223055</v>
       </c>
       <c r="S16" t="n">
-        <v>16630.4480787254</v>
+        <v>16953.02535145267</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -1925,7 +1925,7 @@
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="n">
-        <v>1.724476723897621</v>
+        <v>1.695156758380836</v>
       </c>
     </row>
     <row r="17">
@@ -1989,7 +1989,7 @@
         <v>0.009388620787253983</v>
       </c>
       <c r="P17" t="n">
-        <v>197.2989043506941</v>
+        <v>171.852594747104</v>
       </c>
       <c r="Q17" t="n">
         <v>24884.73840206186</v>
@@ -2007,16 +2007,16 @@
         <v>215.1860689856465</v>
       </c>
       <c r="V17" t="n">
-        <v>13.80550514136005</v>
+        <v>15.84969399156607</v>
       </c>
       <c r="W17" t="n">
-        <v>0.2300917523560008</v>
+        <v>0.2641615665261011</v>
       </c>
       <c r="X17" t="n">
         <v>0.004647140982284977</v>
       </c>
       <c r="Y17" t="n">
-        <v>126.127098799443</v>
+        <v>144.802808701736</v>
       </c>
       <c r="Z17" t="n">
         <v>1.824284824959574</v>
@@ -2083,7 +2083,7 @@
         <v>0.03009892636012183</v>
       </c>
       <c r="P18" t="n">
-        <v>363.0379448902811</v>
+        <v>261.3962064372664</v>
       </c>
       <c r="Q18" t="n">
         <v>18556.36234770384</v>
@@ -2101,16 +2101,16 @@
         <v>96.14235857018933</v>
       </c>
       <c r="V18" t="n">
-        <v>6.990140737158774</v>
+        <v>9.708198761947168</v>
       </c>
       <c r="W18" t="n">
-        <v>0.1165023456193129</v>
+        <v>0.1618033126991195</v>
       </c>
       <c r="X18" t="n">
         <v>0.01040124264550826</v>
       </c>
       <c r="Y18" t="n">
-        <v>51.11411247469469</v>
+        <v>70.9894095274763</v>
       </c>
       <c r="Z18" t="n">
         <v>2.279259875185943</v>
@@ -2177,7 +2177,7 @@
         <v>0.01352985418814433</v>
       </c>
       <c r="P19" t="n">
-        <v>103.2973274500203</v>
+        <v>212.0413838470726</v>
       </c>
       <c r="Q19" t="n">
         <v>18339.46464386129</v>
@@ -2195,16 +2195,16 @@
         <v>78.48157589979928</v>
       </c>
       <c r="V19" t="n">
-        <v>22.25723425430395</v>
+        <v>10.84275518856639</v>
       </c>
       <c r="W19" t="n">
-        <v>0.3709539042383992</v>
+        <v>0.1807125864761065</v>
       </c>
       <c r="X19" t="n">
         <v>0.01274184403836057</v>
       </c>
       <c r="Y19" t="n">
-        <v>177.540553048042</v>
+        <v>86.49002525416449</v>
       </c>
       <c r="Z19" t="n">
         <v>2.089403788992479</v>
@@ -2271,7 +2271,7 @@
         <v>0.02055240276476101</v>
       </c>
       <c r="P20" t="n">
-        <v>47.30726184726024</v>
+        <v>44.28415863123247</v>
       </c>
       <c r="Q20" t="n">
         <v>16801.97029053421</v>
@@ -2289,16 +2289,16 @@
         <v>281.7360333240156</v>
       </c>
       <c r="V20" t="n">
-        <v>47.48366941187022</v>
+        <v>50.72519049174873</v>
       </c>
       <c r="W20" t="n">
-        <v>0.791394490197837</v>
+        <v>0.8454198415291456</v>
       </c>
       <c r="X20" t="n">
         <v>0.003549421734244167</v>
       </c>
       <c r="Y20" t="n">
-        <v>355.166831358414</v>
+        <v>379.4126570282</v>
       </c>
       <c r="Z20" t="n">
         <v>2.22823310152858</v>
@@ -2437,7 +2437,7 @@
         <v>0.007185580093720712</v>
       </c>
       <c r="P22" t="n">
-        <v>93.15932548944448</v>
+        <v>115.3933315841586</v>
       </c>
       <c r="Q22" t="n">
         <v>10267.57471883786</v>
@@ -2455,16 +2455,16 @@
         <v>479.0973514199918</v>
       </c>
       <c r="V22" t="n">
-        <v>22.58336379722525</v>
+        <v>18.23199754916396</v>
       </c>
       <c r="W22" t="n">
-        <v>0.3763893966204208</v>
+        <v>0.3038666258193994</v>
       </c>
       <c r="X22" t="n">
         <v>0.002087258460177478</v>
       </c>
       <c r="Y22" t="n">
-        <v>110.215211036508</v>
+        <v>88.9789260599476</v>
       </c>
       <c r="Z22" t="n">
         <v>3.415040383996947</v>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>K-EXAONE 2.0 0803</t>
+          <t>K-EXAONE 2.0</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2675,7 +2675,7 @@
         <v>0.04498824566541706</v>
       </c>
       <c r="P25" t="n">
-        <v>112.0881023675839</v>
+        <v>105.7984691971073</v>
       </c>
       <c r="Q25" t="n">
         <v>15923.96059044049</v>
@@ -2693,16 +2693,16 @@
         <v>73.58654276566904</v>
       </c>
       <c r="V25" t="n">
-        <v>16.26875197123437</v>
+        <v>17.23591607877827</v>
       </c>
       <c r="W25" t="n">
-        <v>0.2711458661872395</v>
+        <v>0.2872652679796379</v>
       </c>
       <c r="X25" t="n">
         <v>0.01358944125401334</v>
       </c>
       <c r="Y25" t="n">
-        <v>142.06646605738</v>
+        <v>150.512202220747</v>
       </c>
       <c r="Z25" t="n">
         <v>1.908584578134892</v>
@@ -2769,7 +2769,7 @@
         <v>0.02023401440955951</v>
       </c>
       <c r="P26" t="n">
-        <v>107.600891029003</v>
+        <v>148.1824024602097</v>
       </c>
       <c r="Q26" t="n">
         <v>13759.47640581068</v>
@@ -2787,16 +2787,16 @@
         <v>157.9800483099863</v>
       </c>
       <c r="V26" t="n">
-        <v>16.6682273996333</v>
+        <v>12.1034352952685</v>
       </c>
       <c r="W26" t="n">
-        <v>0.2778037899938883</v>
+        <v>0.2017239215878083</v>
       </c>
       <c r="X26" t="n">
         <v>0.006329913243461058</v>
       </c>
       <c r="Y26" t="n">
-        <v>127.875115849198</v>
+        <v>92.85499612213002</v>
       </c>
       <c r="Z26" t="n">
         <v>2.172461687710218</v>
@@ -2863,7 +2863,7 @@
         <v>0.01422300783036551</v>
       </c>
       <c r="P27" t="n">
-        <v>172.4076415513091</v>
+        <v>154.1750937669572</v>
       </c>
       <c r="Q27" t="n">
         <v>27646.50421743205</v>
@@ -2881,16 +2881,16 @@
         <v>161.7135109478305</v>
       </c>
       <c r="V27" t="n">
-        <v>8.396300396451242</v>
+        <v>9.389236054537925</v>
       </c>
       <c r="W27" t="n">
-        <v>0.139938339940854</v>
+        <v>0.1564872675756321</v>
       </c>
       <c r="X27" t="n">
         <v>0.006183775209250168</v>
       </c>
       <c r="Y27" t="n">
-        <v>160.355445783442</v>
+        <v>179.31887402787</v>
       </c>
       <c r="Z27" t="n">
         <v>0.8726759434777098</v>
@@ -2957,7 +2957,7 @@
         <v>0.002903907092783505</v>
       </c>
       <c r="P28" t="n">
-        <v>106.3023063930202</v>
+        <v>111.2793241153015</v>
       </c>
       <c r="Q28" t="n">
         <v>32369.63903467666</v>
@@ -2975,16 +2975,16 @@
         <v>366.5784411818914</v>
       </c>
       <c r="V28" t="n">
-        <v>13.3240218769925</v>
+        <v>12.72809901763773</v>
       </c>
       <c r="W28" t="n">
-        <v>0.2220670312832083</v>
+        <v>0.2121349836272955</v>
       </c>
       <c r="X28" t="n">
         <v>0.002727929107821737</v>
       </c>
       <c r="Y28" t="n">
-        <v>304.505519522783</v>
+        <v>290.886373475247</v>
       </c>
       <c r="Z28" t="n">
         <v>0.7292709558474632</v>
@@ -3051,7 +3051,7 @@
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>54.74174810119658</v>
+        <v>57.59931764497868</v>
       </c>
       <c r="Q29" t="n">
         <v>13793.52434395501</v>
@@ -3067,16 +3067,16 @@
       </c>
       <c r="U29" t="inlineStr"/>
       <c r="V29" t="n">
-        <v>24.9574301443024</v>
+        <v>23.71926283282479</v>
       </c>
       <c r="W29" t="n">
-        <v>0.4159571690717067</v>
+        <v>0.3953210472137465</v>
       </c>
       <c r="X29" t="n">
         <v>0</v>
       </c>
       <c r="Y29" t="n">
-        <v>251.974495196172</v>
+        <v>239.4737456609</v>
       </c>
       <c r="Z29" t="n">
         <v>1.650790762564551</v>

</xml_diff>

<commit_message>
fix: models tab estimates + models_full scrape_date crash
- models_full.html froze at Loading: META lacked scrape_date, template
  called .slice() on undefined. build_index_tab.py now emits it (CSV
  mtime) and template guards for missing key.
- models.html cost/time/token columns were all empty: source page
  models/capabilities/agentic 404s and fallback page carries no
  costPerTask fields. intel_index_full_extract.py now writes full
  per-task estimate breakdowns (cost split, tokens, time) and
  src/main.py backfills the models tab from those estimates (measured
  values would win if the page returns).
- scrape.yml: run extractor before main.py so same-run estimates used.
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Agentic Models" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agentic Models" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z28"/>
+  <dimension ref="A1:Z29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,54 +591,82 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>56.7580864237761</v>
+        <v>53.3737509623252</v>
       </c>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>1.203406</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.051436</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.064901</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1.087069</v>
+      </c>
+      <c r="P2" t="n">
+        <v>213.3</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>23039.4</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1298</v>
+      </c>
+      <c r="S2" t="n">
+        <v>21741.4</v>
+      </c>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
+      <c r="U2" t="n">
+        <v>44.35223936254697</v>
+      </c>
+      <c r="V2" t="n">
+        <v>15.01371335086503</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.2502285558477506</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.02254677586459017</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>108.014064697609</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2.316629381074385</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gpt-6-astra</t>
+          <t>claude-fable-5-1-xhigh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Fable 5.1 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (max)</t>
+          <t>Claude Fable 5.1 (xhigh with fallback)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -653,39 +681,67 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>54.6573323423926</v>
+        <v>53.1840337538944</v>
       </c>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0.556978</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.048158</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.056185</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.452635</v>
+      </c>
+      <c r="P3" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>10176.4</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1123.7</v>
+      </c>
+      <c r="S3" t="n">
+        <v>9052.700000000001</v>
+      </c>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
-      <c r="Z3" t="inlineStr"/>
+      <c r="U3" t="n">
+        <v>95.48677641467778</v>
+      </c>
+      <c r="V3" t="n">
+        <v>30.24684384107738</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.5041140640179563</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0.0104726543040601</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>96.45876777251185</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>5.226212978449589</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gpt-6-astra-xhigh</t>
+          <t>gpt-6-astra</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (xhigh)</t>
+          <t>GPT-6 Astra (max)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -715,54 +771,82 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>54.3148645943349</v>
+        <v>52.814069395513</v>
       </c>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>0.30341</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.022917</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.022384</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.25811</v>
+      </c>
+      <c r="P4" t="n">
+        <v>92.3</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>5609.9</v>
+      </c>
+      <c r="R4" t="n">
+        <v>447.7</v>
+      </c>
+      <c r="S4" t="n">
+        <v>5162.2</v>
+      </c>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
-      <c r="Z4" t="inlineStr"/>
+      <c r="U4" t="n">
+        <v>174.0683213984806</v>
+      </c>
+      <c r="V4" t="n">
+        <v>34.33200610759242</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.572200101793207</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0.005744870703445117</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>60.77898158179848</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>9.414440434858555</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>claude-opus-5</t>
+          <t>gpt-6-astra-xhigh</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (Adaptive Reasoning, Max Effort)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (max)</t>
+          <t>GPT-6 Astra (xhigh)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -777,39 +861,67 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>54.0539443539342</v>
+        <v>52.5059027108782</v>
       </c>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0.172456</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.023073</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.02257</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.126814</v>
+      </c>
+      <c r="P5" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2987.7</v>
+      </c>
+      <c r="R5" t="n">
+        <v>451.4</v>
+      </c>
+      <c r="S5" t="n">
+        <v>2536.3</v>
+      </c>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
+      <c r="U5" t="n">
+        <v>304.4597039875574</v>
+      </c>
+      <c r="V5" t="n">
+        <v>59.89266468921468</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.998211078153578</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.00328450690486406</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>56.80038022813688</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>17.5740210566249</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>claude-fable-5-1-xhigh</t>
+          <t>claude-fable-5-1-high</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (Adaptive Reasoning, Xhigh Effort, Default Fallback)</t>
+          <t>Claude Fable 5.1 (Adaptive Reasoning, High Effort, Default Fallback)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Claude Fable 5.1 (xhigh with fallback)</t>
+          <t>Claude Fable 5.1 (high with fallback)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -839,54 +951,82 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>53.8031695908873</v>
+        <v>51.2094958852237</v>
       </c>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0.214587</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.044761</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.046826</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="P6" t="n">
+        <v>38.2</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>3396.5</v>
+      </c>
+      <c r="R6" t="n">
+        <v>936.5</v>
+      </c>
+      <c r="S6" t="n">
+        <v>2460</v>
+      </c>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
+      <c r="U6" t="n">
+        <v>238.6421166483697</v>
+      </c>
+      <c r="V6" t="n">
+        <v>80.43376317050843</v>
+      </c>
+      <c r="W6" t="n">
+        <v>1.340562719508474</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0.004190375169498949</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>88.91361256544502</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>15.077137019056</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>claude-opus-5-xhigh</t>
+          <t>gpt-6-astra-high</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (Adaptive Reasoning, Xhigh Effort)</t>
+          <t>GPT-6 Astra (high)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Claude Opus 5 (xhigh)</t>
+          <t>GPT-6 Astra (high)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>anthropic</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -901,54 +1041,82 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>53.3699026217041</v>
+        <v>51.0480721636152</v>
       </c>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>0.101844</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.022658</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.022004</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.057183</v>
+      </c>
+      <c r="P7" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1583.7</v>
+      </c>
+      <c r="R7" t="n">
+        <v>440.1</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1143.7</v>
+      </c>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
+      <c r="U7" t="n">
+        <v>501.2378948550253</v>
+      </c>
+      <c r="V7" t="n">
+        <v>113.0215619858639</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1.883692699764399</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0.001995060649373354</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>58.43911439114391</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>32.23342310009168</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gpt-6-astra-high</t>
+          <t>claude-opus-5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (high)</t>
+          <t>Claude Opus 5 (Adaptive Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (high)</t>
+          <t>Claude Opus 5 (max)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>anthropic</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -963,24 +1131,52 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>53.3589099296435</v>
+        <v>50.7001865797629</v>
       </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>0.255456</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.019565</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.02643</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.20946</v>
+      </c>
+      <c r="P8" t="n">
+        <v>111.6</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>9435.6</v>
+      </c>
+      <c r="R8" t="n">
+        <v>1057.2</v>
+      </c>
+      <c r="S8" t="n">
+        <v>8378.4</v>
+      </c>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
+      <c r="U8" t="n">
+        <v>198.4693511984956</v>
+      </c>
+      <c r="V8" t="n">
+        <v>27.25816482782952</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.454302747130492</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0.00503856133937712</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>84.54838709677421</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>5.373286974836035</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1025,54 +1221,82 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>53.1913169443817</v>
+        <v>49.6994452733378</v>
       </c>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>0.520062</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.036048</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.046389</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.437625</v>
+      </c>
+      <c r="P9" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>9680.299999999999</v>
+      </c>
+      <c r="R9" t="n">
+        <v>927.8</v>
+      </c>
+      <c r="S9" t="n">
+        <v>8752.5</v>
+      </c>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
+      <c r="U9" t="n">
+        <v>95.56446207055659</v>
+      </c>
+      <c r="V9" t="n">
+        <v>31.55520334815099</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.5259200558025164</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0.01046414094040195</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>102.437037037037</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>5.134081100104109</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>muse-spark-1-3</t>
+          <t>gpt-6-astra-medium</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>GPT-6 Astra (medium)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Muse Spark 1.3 (max)</t>
+          <t>GPT-6 Astra (medium)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1087,54 +1311,82 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>52.953112358762</v>
+        <v>49.6685363034369</v>
       </c>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>0.070427</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.022736</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.022007</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.025683</v>
+      </c>
+      <c r="P10" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>953.8</v>
+      </c>
+      <c r="R10" t="n">
+        <v>440.1</v>
+      </c>
+      <c r="S10" t="n">
+        <v>513.7</v>
+      </c>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
+      <c r="U10" t="n">
+        <v>705.2485027537294</v>
+      </c>
+      <c r="V10" t="n">
+        <v>176.3379987104269</v>
+      </c>
+      <c r="W10" t="n">
+        <v>2.938966645173781</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0.00141793991209535</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>56.43786982248521</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>52.07437230387598</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gpt-6-astra-medium</t>
+          <t>muse-spark-1-3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (medium)</t>
+          <t>Muse Spark 1.3 (max)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GPT-6 Astra (medium)</t>
+          <t>Muse Spark 1.3 (max)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1149,24 +1401,52 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>52.2467486663733</v>
+        <v>48.1690107719685</v>
       </c>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+      <c r="L11" t="n">
+        <v>0.083136</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.004284</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.003428</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.07542500000000001</v>
+      </c>
+      <c r="P11" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>18553.6</v>
+      </c>
+      <c r="R11" t="n">
+        <v>806.5</v>
+      </c>
+      <c r="S11" t="n">
+        <v>17747</v>
+      </c>
       <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>579.4001488160184</v>
+      </c>
+      <c r="V11" t="n">
+        <v>36.44565758282611</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0.6074276263804351</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0.001725922925707667</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>233.9672131147541</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>2.596208324636109</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1211,54 +1491,82 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>51.2551933761681</v>
+        <v>47.0613568915036</v>
       </c>
       <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>0.126688</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.007634</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.007934999999999999</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.111119</v>
+      </c>
+      <c r="P12" t="n">
+        <v>83.09999999999999</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>5952.7</v>
+      </c>
+      <c r="R12" t="n">
+        <v>396.7</v>
+      </c>
+      <c r="S12" t="n">
+        <v>5555.9</v>
+      </c>
       <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
+      <c r="U12" t="n">
+        <v>371.4744639705702</v>
+      </c>
+      <c r="V12" t="n">
+        <v>33.97931905523726</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0.5663219842539543</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0.002691975080363059</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>71.63297232250301</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>7.905884202379357</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>grok-4-6</t>
+          <t>glm-5-3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Grok 4.6 (high)</t>
+          <t>GLM-5.3 (max)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>SpaceXAI</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>xai</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1270,57 +1578,85 @@
         <v>1</v>
       </c>
       <c r="I13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
-        <v>50.5767541460746</v>
+        <v>44.855717385614</v>
       </c>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>0.15892</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.006115</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.004153</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.148652</v>
+      </c>
+      <c r="P13" t="n">
+        <v>407.9</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>34728.3</v>
+      </c>
+      <c r="R13" t="n">
+        <v>943.8</v>
+      </c>
+      <c r="S13" t="n">
+        <v>33784.5</v>
+      </c>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
+      <c r="U13" t="n">
+        <v>282.253444409854</v>
+      </c>
+      <c r="V13" t="n">
+        <v>6.598046195481344</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0.1099674365913557</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0.003542915134626035</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>85.13924981613141</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>1.291618575790177</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>kimi-k3</t>
+          <t>grok-4-6</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Grok 4.6 (high)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kimi K3 (max)</t>
+          <t>Grok 4.6 (high)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Kimi</t>
+          <t>SpaceXAI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>kimi</t>
+          <t>xai</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1332,57 +1668,85 @@
         <v>1</v>
       </c>
       <c r="I14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>50.2337145305853</v>
+        <v>44.4050073012592</v>
       </c>
       <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>0.066873</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.005686</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.003091</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.058096</v>
+      </c>
+      <c r="P14" t="n">
+        <v>180.9</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>10197.8</v>
+      </c>
+      <c r="R14" t="n">
+        <v>515.2</v>
+      </c>
+      <c r="S14" t="n">
+        <v>9682.6</v>
+      </c>
       <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
+      <c r="U14" t="n">
+        <v>664.0199677187983</v>
+      </c>
+      <c r="V14" t="n">
+        <v>14.72802895564152</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0.2454671492606921</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0.001505978808793117</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>56.37258153676063</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>4.354371266475043</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>glm-5-3</t>
+          <t>kimi-k3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GLM-5.3 (max)</t>
+          <t>Kimi K3 (max)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Kimi</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>kimi</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1397,54 +1761,82 @@
         <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>48.5840319700216</v>
+        <v>43.7841729518782</v>
       </c>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>0.163338</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.007471</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.007591</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.148276</v>
+      </c>
+      <c r="P15" t="n">
+        <v>241.1</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>10391.2</v>
+      </c>
+      <c r="R15" t="n">
+        <v>506.1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>9885.1</v>
+      </c>
       <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr"/>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
+      <c r="U15" t="n">
+        <v>268.0587061913222</v>
+      </c>
+      <c r="V15" t="n">
+        <v>10.89610276695434</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0.1816017127825724</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0.003730526100824598</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>43.09912899211945</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>4.213581968577084</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>gemini-3-8-flash</t>
+          <t>gpt-5-6-terra</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GPT-5.6 Terra (max)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Gemini 3.8 Flash (high)</t>
+          <t>GPT-5.6 Terra (max)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1459,54 +1851,82 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>47.0713231150669</v>
+        <v>42.2514998239494</v>
       </c>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>0.14583</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.004243</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.004487</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.137101</v>
+      </c>
+      <c r="P16" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>11799</v>
+      </c>
+      <c r="R16" t="n">
+        <v>373.9</v>
+      </c>
+      <c r="S16" t="n">
+        <v>11425.1</v>
+      </c>
       <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
+      <c r="U16" t="n">
+        <v>289.7311926486279</v>
+      </c>
+      <c r="V16" t="n">
+        <v>24.56482547904035</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0.4094137579840058</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0.003451475109940102</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>114.3313953488372</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>3.58093904771162</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>gpt-5-6-terra</t>
+          <t>glm-5-3-flash</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GPT-5.6 Terra (max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GPT-5.6 Terra (max)</t>
+          <t>GLM-5.3-Flash</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Z AI</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>zai</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1518,57 +1938,85 @@
         <v>1</v>
       </c>
       <c r="I17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
-        <v>46.76875579302</v>
+        <v>41.907366113455</v>
       </c>
       <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>0.022786</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.000576</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.000417</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.021793</v>
+      </c>
+      <c r="P17" t="n">
+        <v>580</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>44420.3</v>
+      </c>
+      <c r="R17" t="n">
+        <v>834.1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>43586.3</v>
+      </c>
       <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
+      <c r="U17" t="n">
+        <v>1839.171689346748</v>
+      </c>
+      <c r="V17" t="n">
+        <v>4.335244770357414</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0.07225407950595689</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0.0005437230280307263</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>76.58672413793104</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.9434282549522401</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>qwen3-8-2-4t-a95b</t>
+          <t>gemini-3-8-flash</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Qwen3.8 2.4T A95B</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Qwen3.8 2.4T A95B</t>
+          <t>Gemini 3.8 Flash (high)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1580,57 +2028,85 @@
         <v>1</v>
       </c>
       <c r="I18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>46.7402728105642</v>
+        <v>41.1863571765904</v>
       </c>
       <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
-      <c r="S18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>0.093127</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.001995</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.002368</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.088764</v>
+      </c>
+      <c r="P18" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>24301.8</v>
+      </c>
+      <c r="R18" t="n">
+        <v>631.5</v>
+      </c>
+      <c r="S18" t="n">
+        <v>23670.3</v>
+      </c>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
+      <c r="U18" t="n">
+        <v>442.2601090617157</v>
+      </c>
+      <c r="V18" t="n">
+        <v>30.77436401737763</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0.5129060669562939</v>
+      </c>
+      <c r="X18" t="n">
+        <v>0.00226111281463202</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>302.6376089663761</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>1.694786278242369</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>glm-5-3-flash</t>
+          <t>qwen3-8-2-4t-a95b</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Qwen3.8 2.4T A95B</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash</t>
+          <t>Qwen3.8 2.4T A95B</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Z AI</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>zai</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1645,24 +2121,52 @@
         <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>46.2237224739457</v>
+        <v>40.0445723105325</v>
       </c>
       <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
-      <c r="S19" t="inlineStr"/>
+      <c r="L19" t="n">
+        <v>0.178757</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.009473000000000001</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.009109000000000001</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.160175</v>
+      </c>
+      <c r="P19" t="n">
+        <v>536.9</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>28213.9</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1518.1</v>
+      </c>
+      <c r="S19" t="n">
+        <v>26695.8</v>
+      </c>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
+      <c r="U19" t="n">
+        <v>224.0168066734869</v>
+      </c>
+      <c r="V19" t="n">
+        <v>4.475087239023934</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0.07458478731706557</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0.004463950784985246</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>52.54963680387409</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>1.419320700453766</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1707,24 +2211,52 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>43.4414655969671</v>
+        <v>37.5048489690841</v>
       </c>
       <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
+      <c r="L20" t="n">
+        <v>0.016448</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.000637</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.000541</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.015269</v>
+      </c>
+      <c r="P20" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>13175.4</v>
+      </c>
+      <c r="R20" t="n">
+        <v>451.2</v>
+      </c>
+      <c r="S20" t="n">
+        <v>12724.3</v>
+      </c>
       <c r="T20" t="inlineStr"/>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
+      <c r="U20" t="n">
+        <v>2280.207257361631</v>
+      </c>
+      <c r="V20" t="n">
+        <v>20.87468402731954</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0.3479114004553256</v>
+      </c>
+      <c r="X20" t="n">
+        <v>0.0004385566253995149</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>122.2207792207792</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>2.846581429716297</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1769,24 +2301,52 @@
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>42.1132549231516</v>
+        <v>36.2828791278402</v>
       </c>
       <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
-      <c r="S21" t="inlineStr"/>
+      <c r="L21" t="n">
+        <v>0.101663</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.003745</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.001918</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.096</v>
+      </c>
+      <c r="P21" t="n">
+        <v>247.7</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>24726.8</v>
+      </c>
+      <c r="R21" t="n">
+        <v>484.3</v>
+      </c>
+      <c r="S21" t="n">
+        <v>24242.5</v>
+      </c>
       <c r="T21" t="inlineStr"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
+      <c r="U21" t="n">
+        <v>356.8936498808829</v>
+      </c>
+      <c r="V21" t="n">
+        <v>8.788747467381558</v>
+      </c>
+      <c r="W21" t="n">
+        <v>0.1464791244563593</v>
+      </c>
+      <c r="X21" t="n">
+        <v>0.002801955149198538</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>99.8255954784013</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>1.467350369956492</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1831,54 +2391,82 @@
         <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>41.4059480116377</v>
+        <v>33.9015108057476</v>
       </c>
       <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
+      <c r="L22" t="n">
+        <v>0.09057999999999999</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.001883</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.003858</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.084838</v>
+      </c>
+      <c r="P22" t="n">
+        <v>490.5</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>29565.5</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1286.1</v>
+      </c>
+      <c r="S22" t="n">
+        <v>28279.4</v>
+      </c>
       <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
+      <c r="U22" t="n">
+        <v>374.2714816267123</v>
+      </c>
+      <c r="V22" t="n">
+        <v>4.146973798868207</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0.0691162299811368</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0.00267185732574028</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>60.27624872579001</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>1.146657787142027</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>k2-horizon-375b-a23b</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>K2 Horizon 375B A23B</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MBZUAI Institute of Foundation Models</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>mbzuai</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1893,54 +2481,82 @@
         <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>37.7506901831038</v>
+        <v>29.6125932236316</v>
       </c>
       <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
+      <c r="L23" t="n">
+        <v>0.026465</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.004611</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.00061</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.021244</v>
+      </c>
+      <c r="P23" t="n">
+        <v>177.6</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>18211.1</v>
+      </c>
+      <c r="R23" t="n">
+        <v>508</v>
+      </c>
+      <c r="S23" t="n">
+        <v>17703.1</v>
+      </c>
       <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
+      <c r="U23" t="n">
+        <v>1118.934185665279</v>
+      </c>
+      <c r="V23" t="n">
+        <v>10.00425446744311</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0.1667375744573851</v>
+      </c>
+      <c r="X23" t="n">
+        <v>0.0008937076128435877</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>102.5399774774775</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>1.626073835387846</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Inkling</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1955,54 +2571,82 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>35.7477256720963</v>
+        <v>25.5423060999384</v>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
+      <c r="L24" t="n">
+        <v>0.09468799999999999</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.002374</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.001895</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.09042</v>
+      </c>
+      <c r="P24" t="n">
+        <v>328.9</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>22793.6</v>
+      </c>
+      <c r="R24" t="n">
+        <v>467.8</v>
+      </c>
+      <c r="S24" t="n">
+        <v>22325.9</v>
+      </c>
       <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
+      <c r="U24" t="n">
+        <v>269.7523033535232</v>
+      </c>
+      <c r="V24" t="n">
+        <v>4.659587613245072</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.07765979355408453</v>
+      </c>
+      <c r="X24" t="n">
+        <v>0.003707104582864127</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>69.30252356339312</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>1.12059113522824</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Inkling</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2017,24 +2661,52 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>32.1665277396553</v>
+        <v>23.4145123422858</v>
       </c>
       <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>0.034269</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.001525</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.002978</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.029765</v>
+      </c>
+      <c r="P25" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>12593.6</v>
+      </c>
+      <c r="R25" t="n">
+        <v>1145.5</v>
+      </c>
+      <c r="S25" t="n">
+        <v>11448.1</v>
+      </c>
       <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>683.2563641275146</v>
+      </c>
+      <c r="V25" t="n">
+        <v>19.48503107541121</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.3247505179235201</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0.00146357948861106</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>174.6685159500694</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>1.859239005708122</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2079,24 +2751,52 @@
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>27.5743377606185</v>
+        <v>22.6606674839812</v>
       </c>
       <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>0.019232</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.000782</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0.001426</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.017024</v>
+      </c>
+      <c r="P26" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>7379.9</v>
+      </c>
+      <c r="R26" t="n">
+        <v>570.5</v>
+      </c>
+      <c r="S26" t="n">
+        <v>6809.5</v>
+      </c>
       <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
+      <c r="U26" t="n">
+        <v>1178.279299291868</v>
+      </c>
+      <c r="V26" t="n">
+        <v>66.97734231718582</v>
+      </c>
+      <c r="W26" t="n">
+        <v>1.116289038619763</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0.000848695212248054</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>363.5418719211822</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>3.070592756538869</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2141,86 +2841,232 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>24.3772708027605</v>
+        <v>18.0678176089465</v>
       </c>
       <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>0.012326</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.00072</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.00067</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.010936</v>
+      </c>
+      <c r="P27" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>7737.1</v>
+      </c>
+      <c r="R27" t="n">
+        <v>446.4</v>
+      </c>
+      <c r="S27" t="n">
+        <v>7290.7</v>
+      </c>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
+      <c r="U27" t="n">
+        <v>1465.829758960449</v>
+      </c>
+      <c r="V27" t="n">
+        <v>14.41581192203178</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0.240263532033863</v>
+      </c>
+      <c r="X27" t="n">
+        <v>0.0006822074622834709</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>102.8869680851064</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>2.335218312926871</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>mistral-medium-3-5</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Mistral Medium 3.5</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Mistral Medium 3.5</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Mistral</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H28" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" t="b">
+        <v>1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>14.8946727802691</v>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>0.108206</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.002141</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.058389</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.047676</v>
+      </c>
+      <c r="P28" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>14142</v>
+      </c>
+      <c r="R28" t="n">
+        <v>7785.3</v>
+      </c>
+      <c r="S28" t="n">
+        <v>6356.8</v>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="n">
+        <v>137.6510801644003</v>
+      </c>
+      <c r="V28" t="n">
+        <v>10.57609901557569</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.1762683169262615</v>
+      </c>
+      <c r="X28" t="n">
+        <v>0.007264745026378824</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>167.3609467455621</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>1.053222513100629</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>gpt-oss-120b</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>gpt-oss-120b (high)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>gpt-oss-120b (high)</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>openai</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>2025-08-05</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="H28" t="b">
-        <v>1</v>
-      </c>
-      <c r="I28" t="b">
-        <v>1</v>
-      </c>
-      <c r="J28" t="n">
-        <v>15.5719877600873</v>
-      </c>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" t="b">
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>12.3483931512592</v>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>0.007271</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.000449</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.000691</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.006131</v>
+      </c>
+      <c r="P29" t="n">
+        <v>50.9</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>11465.4</v>
+      </c>
+      <c r="R29" t="n">
+        <v>1161.3</v>
+      </c>
+      <c r="S29" t="n">
+        <v>10304</v>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="n">
+        <v>1698.307406307138</v>
+      </c>
+      <c r="V29" t="n">
+        <v>14.55606265374366</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.2426010442290609</v>
+      </c>
+      <c r="X29" t="n">
+        <v>0.000588821550377877</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>225.2534381139489</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>1.077013724009559</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-08)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agentic Models" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Agentic Models" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore: update coding-agents leaderboard (2026-09-13)
</commit_message>
<xml_diff>
--- a/data/artificial_analysis_agentic_models.xlsx
+++ b/data/artificial_analysis_agentic_models.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z29"/>
+  <dimension ref="A1:Z31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -607,7 +607,7 @@
         <v>1.087069</v>
       </c>
       <c r="P2" t="n">
-        <v>213.3</v>
+        <v>215</v>
       </c>
       <c r="Q2" t="n">
         <v>23039.4</v>
@@ -623,16 +623,16 @@
         <v>44.35223936254697</v>
       </c>
       <c r="V2" t="n">
-        <v>15.01371335086503</v>
+        <v>14.89500026855587</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2502285558477506</v>
+        <v>0.2482500044759312</v>
       </c>
       <c r="X2" t="n">
         <v>0.02254677586459017</v>
       </c>
       <c r="Y2" t="n">
-        <v>108.014064697609</v>
+        <v>107.16</v>
       </c>
       <c r="Z2" t="n">
         <v>2.316629381074385</v>
@@ -697,7 +697,7 @@
         <v>0.452635</v>
       </c>
       <c r="P3" t="n">
-        <v>105.5</v>
+        <v>105.7</v>
       </c>
       <c r="Q3" t="n">
         <v>10176.4</v>
@@ -713,16 +713,16 @@
         <v>95.48677641467778</v>
       </c>
       <c r="V3" t="n">
-        <v>30.24684384107738</v>
+        <v>30.18961234847364</v>
       </c>
       <c r="W3" t="n">
-        <v>0.5041140640179563</v>
+        <v>0.503160205807894</v>
       </c>
       <c r="X3" t="n">
         <v>0.0104726543040601</v>
       </c>
       <c r="Y3" t="n">
-        <v>96.45876777251185</v>
+        <v>96.27625354777672</v>
       </c>
       <c r="Z3" t="n">
         <v>5.226212978449589</v>
@@ -787,7 +787,7 @@
         <v>0.25811</v>
       </c>
       <c r="P4" t="n">
-        <v>92.3</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="Q4" t="n">
         <v>5609.9</v>
@@ -803,16 +803,16 @@
         <v>174.0683213984806</v>
       </c>
       <c r="V4" t="n">
-        <v>34.33200610759242</v>
+        <v>34.036994239858</v>
       </c>
       <c r="W4" t="n">
-        <v>0.572200101793207</v>
+        <v>0.5672832373309667</v>
       </c>
       <c r="X4" t="n">
         <v>0.005744870703445117</v>
       </c>
       <c r="Y4" t="n">
-        <v>60.77898158179848</v>
+        <v>60.25671321160043</v>
       </c>
       <c r="Z4" t="n">
         <v>9.414440434858555</v>
@@ -877,7 +877,7 @@
         <v>0.126814</v>
       </c>
       <c r="P5" t="n">
-        <v>52.6</v>
+        <v>58.6</v>
       </c>
       <c r="Q5" t="n">
         <v>2987.7</v>
@@ -893,16 +893,16 @@
         <v>304.4597039875574</v>
       </c>
       <c r="V5" t="n">
-        <v>59.89266468921468</v>
+        <v>53.76030994287871</v>
       </c>
       <c r="W5" t="n">
-        <v>0.998211078153578</v>
+        <v>0.8960051657146451</v>
       </c>
       <c r="X5" t="n">
         <v>0.00328450690486406</v>
       </c>
       <c r="Y5" t="n">
-        <v>56.80038022813688</v>
+        <v>50.98464163822525</v>
       </c>
       <c r="Z5" t="n">
         <v>17.5740210566249</v>
@@ -967,7 +967,7 @@
         <v>0.123</v>
       </c>
       <c r="P6" t="n">
-        <v>38.2</v>
+        <v>40.6</v>
       </c>
       <c r="Q6" t="n">
         <v>3396.5</v>
@@ -983,16 +983,16 @@
         <v>238.6421166483697</v>
       </c>
       <c r="V6" t="n">
-        <v>80.43376317050843</v>
+        <v>75.67905795845867</v>
       </c>
       <c r="W6" t="n">
-        <v>1.340562719508474</v>
+        <v>1.261317632640978</v>
       </c>
       <c r="X6" t="n">
         <v>0.004190375169498949</v>
       </c>
       <c r="Y6" t="n">
-        <v>88.91361256544502</v>
+        <v>83.6576354679803</v>
       </c>
       <c r="Z6" t="n">
         <v>15.077137019056</v>
@@ -1057,7 +1057,7 @@
         <v>0.057183</v>
       </c>
       <c r="P7" t="n">
-        <v>27.1</v>
+        <v>31</v>
       </c>
       <c r="Q7" t="n">
         <v>1583.7</v>
@@ -1073,16 +1073,16 @@
         <v>501.2378948550253</v>
       </c>
       <c r="V7" t="n">
-        <v>113.0215619858639</v>
+        <v>98.80272031667458</v>
       </c>
       <c r="W7" t="n">
-        <v>1.883692699764399</v>
+        <v>1.64671200527791</v>
       </c>
       <c r="X7" t="n">
         <v>0.001995060649373354</v>
       </c>
       <c r="Y7" t="n">
-        <v>58.43911439114391</v>
+        <v>51.08709677419355</v>
       </c>
       <c r="Z7" t="n">
         <v>32.23342310009168</v>
@@ -1147,7 +1147,7 @@
         <v>0.20946</v>
       </c>
       <c r="P8" t="n">
-        <v>111.6</v>
+        <v>109.3</v>
       </c>
       <c r="Q8" t="n">
         <v>9435.6</v>
@@ -1163,16 +1163,16 @@
         <v>198.4693511984956</v>
       </c>
       <c r="V8" t="n">
-        <v>27.25816482782952</v>
+        <v>27.83175841524039</v>
       </c>
       <c r="W8" t="n">
-        <v>0.454302747130492</v>
+        <v>0.4638626402540064</v>
       </c>
       <c r="X8" t="n">
         <v>0.00503856133937712</v>
       </c>
       <c r="Y8" t="n">
-        <v>84.54838709677421</v>
+        <v>86.32753888380604</v>
       </c>
       <c r="Z8" t="n">
         <v>5.373286974836035</v>
@@ -1237,7 +1237,7 @@
         <v>0.437625</v>
       </c>
       <c r="P9" t="n">
-        <v>94.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="Q9" t="n">
         <v>9680.299999999999</v>
@@ -1253,16 +1253,16 @@
         <v>95.56446207055659</v>
       </c>
       <c r="V9" t="n">
-        <v>31.55520334815099</v>
+        <v>31.92683850535618</v>
       </c>
       <c r="W9" t="n">
-        <v>0.5259200558025164</v>
+        <v>0.5321139750892698</v>
       </c>
       <c r="X9" t="n">
         <v>0.01046414094040195</v>
       </c>
       <c r="Y9" t="n">
-        <v>102.437037037037</v>
+        <v>103.6434689507495</v>
       </c>
       <c r="Z9" t="n">
         <v>5.134081100104109</v>
@@ -1327,7 +1327,7 @@
         <v>0.025683</v>
       </c>
       <c r="P10" t="n">
-        <v>16.9</v>
+        <v>18.9</v>
       </c>
       <c r="Q10" t="n">
         <v>953.8</v>
@@ -1343,16 +1343,16 @@
         <v>705.2485027537294</v>
       </c>
       <c r="V10" t="n">
-        <v>176.3379987104269</v>
+        <v>157.6778930267838</v>
       </c>
       <c r="W10" t="n">
-        <v>2.938966645173781</v>
+        <v>2.62796488377973</v>
       </c>
       <c r="X10" t="n">
         <v>0.00141793991209535</v>
       </c>
       <c r="Y10" t="n">
-        <v>56.43786982248521</v>
+        <v>50.46560846560847</v>
       </c>
       <c r="Z10" t="n">
         <v>52.07437230387598</v>
@@ -1417,7 +1417,7 @@
         <v>0.07542500000000001</v>
       </c>
       <c r="P11" t="n">
-        <v>79.3</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="Q11" t="n">
         <v>18553.6</v>
@@ -1433,16 +1433,16 @@
         <v>579.4001488160184</v>
       </c>
       <c r="V11" t="n">
-        <v>36.44565758282611</v>
+        <v>38.58665749423378</v>
       </c>
       <c r="W11" t="n">
-        <v>0.6074276263804351</v>
+        <v>0.6431109582372296</v>
       </c>
       <c r="X11" t="n">
         <v>0.001725922925707667</v>
       </c>
       <c r="Y11" t="n">
-        <v>233.9672131147541</v>
+        <v>247.7116154873164</v>
       </c>
       <c r="Z11" t="n">
         <v>2.596208324636109</v>
@@ -1507,7 +1507,7 @@
         <v>0.111119</v>
       </c>
       <c r="P12" t="n">
-        <v>83.09999999999999</v>
+        <v>96.2</v>
       </c>
       <c r="Q12" t="n">
         <v>5952.7</v>
@@ -1523,16 +1523,16 @@
         <v>371.4744639705702</v>
       </c>
       <c r="V12" t="n">
-        <v>33.97931905523726</v>
+        <v>29.35219764542844</v>
       </c>
       <c r="W12" t="n">
-        <v>0.5663219842539543</v>
+        <v>0.489203294090474</v>
       </c>
       <c r="X12" t="n">
         <v>0.002691975080363059</v>
       </c>
       <c r="Y12" t="n">
-        <v>71.63297232250301</v>
+        <v>61.87837837837837</v>
       </c>
       <c r="Z12" t="n">
         <v>7.905884202379357</v>
@@ -1597,7 +1597,7 @@
         <v>0.148652</v>
       </c>
       <c r="P13" t="n">
-        <v>407.9</v>
+        <v>407.1</v>
       </c>
       <c r="Q13" t="n">
         <v>34728.3</v>
@@ -1613,16 +1613,16 @@
         <v>282.253444409854</v>
       </c>
       <c r="V13" t="n">
-        <v>6.598046195481344</v>
+        <v>6.611012142315991</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1099674365913557</v>
+        <v>0.1101835357052665</v>
       </c>
       <c r="X13" t="n">
         <v>0.003542915134626035</v>
       </c>
       <c r="Y13" t="n">
-        <v>85.13924981613141</v>
+        <v>85.30655858511423</v>
       </c>
       <c r="Z13" t="n">
         <v>1.291618575790177</v>
@@ -1687,7 +1687,7 @@
         <v>0.058096</v>
       </c>
       <c r="P14" t="n">
-        <v>180.9</v>
+        <v>174</v>
       </c>
       <c r="Q14" t="n">
         <v>10197.8</v>
@@ -1703,16 +1703,16 @@
         <v>664.0199677187983</v>
       </c>
       <c r="V14" t="n">
-        <v>14.72802895564152</v>
+        <v>15.31207148319283</v>
       </c>
       <c r="W14" t="n">
-        <v>0.2454671492606921</v>
+        <v>0.2552011913865471</v>
       </c>
       <c r="X14" t="n">
         <v>0.001505978808793117</v>
       </c>
       <c r="Y14" t="n">
-        <v>56.37258153676063</v>
+        <v>58.60804597701149</v>
       </c>
       <c r="Z14" t="n">
         <v>4.354371266475043</v>
@@ -1777,7 +1777,7 @@
         <v>0.148276</v>
       </c>
       <c r="P15" t="n">
-        <v>241.1</v>
+        <v>265.4</v>
       </c>
       <c r="Q15" t="n">
         <v>10391.2</v>
@@ -1793,16 +1793,16 @@
         <v>268.0587061913222</v>
       </c>
       <c r="V15" t="n">
-        <v>10.89610276695434</v>
+        <v>9.898456582941568</v>
       </c>
       <c r="W15" t="n">
-        <v>0.1816017127825724</v>
+        <v>0.1649742763823595</v>
       </c>
       <c r="X15" t="n">
         <v>0.003730526100824598</v>
       </c>
       <c r="Y15" t="n">
-        <v>43.09912899211945</v>
+        <v>39.15297663903542</v>
       </c>
       <c r="Z15" t="n">
         <v>4.213581968577084</v>
@@ -1867,7 +1867,7 @@
         <v>0.137101</v>
       </c>
       <c r="P16" t="n">
-        <v>103.2</v>
+        <v>109.6</v>
       </c>
       <c r="Q16" t="n">
         <v>11799</v>
@@ -1883,16 +1883,16 @@
         <v>289.7311926486279</v>
       </c>
       <c r="V16" t="n">
-        <v>24.56482547904035</v>
+        <v>23.13038311530077</v>
       </c>
       <c r="W16" t="n">
-        <v>0.4094137579840058</v>
+        <v>0.3855063852550128</v>
       </c>
       <c r="X16" t="n">
         <v>0.003451475109940102</v>
       </c>
       <c r="Y16" t="n">
-        <v>114.3313953488372</v>
+        <v>107.6551094890511</v>
       </c>
       <c r="Z16" t="n">
         <v>3.58093904771162</v>
@@ -1957,7 +1957,7 @@
         <v>0.021793</v>
       </c>
       <c r="P17" t="n">
-        <v>580</v>
+        <v>334.9</v>
       </c>
       <c r="Q17" t="n">
         <v>44420.3</v>
@@ -1973,16 +1973,16 @@
         <v>1839.171689346748</v>
       </c>
       <c r="V17" t="n">
-        <v>4.335244770357414</v>
+        <v>7.508038121252016</v>
       </c>
       <c r="W17" t="n">
-        <v>0.07225407950595689</v>
+        <v>0.1251339686875336</v>
       </c>
       <c r="X17" t="n">
         <v>0.0005437230280307263</v>
       </c>
       <c r="Y17" t="n">
-        <v>76.58672413793104</v>
+        <v>132.6375037324575</v>
       </c>
       <c r="Z17" t="n">
         <v>0.9434282549522401</v>
@@ -2047,7 +2047,7 @@
         <v>0.088764</v>
       </c>
       <c r="P18" t="n">
-        <v>80.3</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="Q18" t="n">
         <v>24301.8</v>
@@ -2063,16 +2063,16 @@
         <v>442.2601090617157</v>
       </c>
       <c r="V18" t="n">
-        <v>30.77436401737763</v>
+        <v>30.28408615925765</v>
       </c>
       <c r="W18" t="n">
-        <v>0.5129060669562939</v>
+        <v>0.5047347693209608</v>
       </c>
       <c r="X18" t="n">
         <v>0.00226111281463202</v>
       </c>
       <c r="Y18" t="n">
-        <v>302.6376089663761</v>
+        <v>297.8161764705882</v>
       </c>
       <c r="Z18" t="n">
         <v>1.694786278242369</v>
@@ -2137,7 +2137,7 @@
         <v>0.160175</v>
       </c>
       <c r="P19" t="n">
-        <v>536.9</v>
+        <v>617.9</v>
       </c>
       <c r="Q19" t="n">
         <v>28213.9</v>
@@ -2153,16 +2153,16 @@
         <v>224.0168066734869</v>
       </c>
       <c r="V19" t="n">
-        <v>4.475087239023934</v>
+        <v>3.888451753733533</v>
       </c>
       <c r="W19" t="n">
-        <v>0.07458478731706557</v>
+        <v>0.06480752922889223</v>
       </c>
       <c r="X19" t="n">
         <v>0.004463950784985246</v>
       </c>
       <c r="Y19" t="n">
-        <v>52.54963680387409</v>
+        <v>45.66094837352323</v>
       </c>
       <c r="Z19" t="n">
         <v>1.419320700453766</v>
@@ -2171,217 +2171,217 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>gpt-5-6-luna</t>
+          <t>deepseek-v4-1-flash</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>DeepSeek V4.1 Flash (Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GPT-5.6 Luna (max)</t>
+          <t>DeepSeek V4.1 Flash (max)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H20" t="b">
         <v>1</v>
       </c>
       <c r="I20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>37.5048489690841</v>
+        <v>39.545442472527</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
-        <v>0.016448</v>
+        <v>0.027666</v>
       </c>
       <c r="M20" t="n">
-        <v>0.000637</v>
+        <v>0.000862</v>
       </c>
       <c r="N20" t="n">
-        <v>0.000541</v>
+        <v>0.000595</v>
       </c>
       <c r="O20" t="n">
-        <v>0.015269</v>
+        <v>0.02621</v>
       </c>
       <c r="P20" t="n">
-        <v>107.8</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="Q20" t="n">
-        <v>13175.4</v>
+        <v>22336.9</v>
       </c>
       <c r="R20" t="n">
-        <v>451.2</v>
+        <v>495.4</v>
       </c>
       <c r="S20" t="n">
-        <v>12724.3</v>
+        <v>21841.5</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="n">
-        <v>2280.207257361631</v>
+        <v>1429.387785459662</v>
       </c>
       <c r="V20" t="n">
-        <v>20.87468402731954</v>
+        <v>30.5763730457683</v>
       </c>
       <c r="W20" t="n">
-        <v>0.3479114004553256</v>
+        <v>0.5096062174294717</v>
       </c>
       <c r="X20" t="n">
-        <v>0.0004385566253995149</v>
+        <v>0.0006996002135826427</v>
       </c>
       <c r="Y20" t="n">
-        <v>122.2207792207792</v>
+        <v>287.8466494845361</v>
       </c>
       <c r="Z20" t="n">
-        <v>2.846581429716297</v>
+        <v>1.770408717079228</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>deepseek-v4-pro</t>
+          <t>gpt-5-6-luna</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro 0813 (Reasoning, Max Effort)</t>
+          <t>GPT-5.6 Luna (max)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Pro 0813 (max)</t>
+          <t>GPT-5.6 Luna (max)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>DeepSeek</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>deepseek</t>
+          <t>openai</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
       </c>
       <c r="I21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>36.2828791278402</v>
+        <v>37.5048489690841</v>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
-        <v>0.101663</v>
+        <v>0.016448</v>
       </c>
       <c r="M21" t="n">
-        <v>0.003745</v>
+        <v>0.000637</v>
       </c>
       <c r="N21" t="n">
-        <v>0.001918</v>
+        <v>0.000541</v>
       </c>
       <c r="O21" t="n">
-        <v>0.096</v>
+        <v>0.015269</v>
       </c>
       <c r="P21" t="n">
-        <v>247.7</v>
+        <v>112.5</v>
       </c>
       <c r="Q21" t="n">
-        <v>24726.8</v>
+        <v>13175.4</v>
       </c>
       <c r="R21" t="n">
-        <v>484.3</v>
+        <v>451.2</v>
       </c>
       <c r="S21" t="n">
-        <v>24242.5</v>
+        <v>12724.3</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="n">
-        <v>356.8936498808829</v>
+        <v>2280.207257361631</v>
       </c>
       <c r="V21" t="n">
-        <v>8.788747467381558</v>
+        <v>20.00258611684485</v>
       </c>
       <c r="W21" t="n">
-        <v>0.1464791244563593</v>
+        <v>0.3333764352807476</v>
       </c>
       <c r="X21" t="n">
-        <v>0.002801955149198538</v>
+        <v>0.0004385566253995149</v>
       </c>
       <c r="Y21" t="n">
-        <v>99.8255954784013</v>
+        <v>117.1146666666667</v>
       </c>
       <c r="Z21" t="n">
-        <v>1.467350369956492</v>
+        <v>2.846581429716297</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>qwen3-8-27b</t>
+          <t>deepseek-v4-pro</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>DeepSeek V4 Pro 0813 (Reasoning, Max Effort)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Qwen3.8 27B (xhigh)</t>
+          <t>DeepSeek V4 Pro 0813 (max)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>DeepSeek</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>alibaba</t>
+          <t>deepseek</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H22" t="b">
@@ -2391,87 +2391,87 @@
         <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>33.9015108057476</v>
+        <v>36.2828791278402</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
-        <v>0.09057999999999999</v>
+        <v>0.101663</v>
       </c>
       <c r="M22" t="n">
-        <v>0.001883</v>
+        <v>0.003745</v>
       </c>
       <c r="N22" t="n">
-        <v>0.003858</v>
+        <v>0.001918</v>
       </c>
       <c r="O22" t="n">
-        <v>0.084838</v>
+        <v>0.096</v>
       </c>
       <c r="P22" t="n">
-        <v>490.5</v>
+        <v>282.1</v>
       </c>
       <c r="Q22" t="n">
-        <v>29565.5</v>
+        <v>24726.8</v>
       </c>
       <c r="R22" t="n">
-        <v>1286.1</v>
+        <v>484.3</v>
       </c>
       <c r="S22" t="n">
-        <v>28279.4</v>
+        <v>24242.5</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="n">
-        <v>374.2714816267123</v>
+        <v>356.8936498808829</v>
       </c>
       <c r="V22" t="n">
-        <v>4.146973798868207</v>
+        <v>7.717024982879871</v>
       </c>
       <c r="W22" t="n">
-        <v>0.0691162299811368</v>
+        <v>0.1286170830479978</v>
       </c>
       <c r="X22" t="n">
-        <v>0.00267185732574028</v>
+        <v>0.002801955149198538</v>
       </c>
       <c r="Y22" t="n">
-        <v>60.27624872579001</v>
+        <v>87.65260545905706</v>
       </c>
       <c r="Z22" t="n">
-        <v>1.146657787142027</v>
+        <v>1.467350369956492</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>qwen3-8-27b</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MiniMax-M3</t>
+          <t>Qwen3.8 27B (xhigh)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MiniMax</t>
+          <t>Alibaba</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>minimax</t>
+          <t>alibaba</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>large</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -2481,82 +2481,82 @@
         <v>1</v>
       </c>
       <c r="J23" t="n">
-        <v>29.6125932236316</v>
+        <v>33.9015108057476</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
-        <v>0.026465</v>
+        <v>0.09057999999999999</v>
       </c>
       <c r="M23" t="n">
-        <v>0.004611</v>
+        <v>0.001883</v>
       </c>
       <c r="N23" t="n">
-        <v>0.00061</v>
+        <v>0.003858</v>
       </c>
       <c r="O23" t="n">
-        <v>0.021244</v>
+        <v>0.084838</v>
       </c>
       <c r="P23" t="n">
-        <v>177.6</v>
+        <v>560.6</v>
       </c>
       <c r="Q23" t="n">
-        <v>18211.1</v>
+        <v>29565.5</v>
       </c>
       <c r="R23" t="n">
-        <v>508</v>
+        <v>1286.1</v>
       </c>
       <c r="S23" t="n">
-        <v>17703.1</v>
+        <v>28279.4</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="n">
-        <v>1118.934185665279</v>
+        <v>374.2714816267123</v>
       </c>
       <c r="V23" t="n">
-        <v>10.00425446744311</v>
+        <v>3.628417139395034</v>
       </c>
       <c r="W23" t="n">
-        <v>0.1667375744573851</v>
+        <v>0.06047361898991722</v>
       </c>
       <c r="X23" t="n">
-        <v>0.0008937076128435877</v>
+        <v>0.00267185732574028</v>
       </c>
       <c r="Y23" t="n">
-        <v>102.5399774774775</v>
+        <v>52.73902961113093</v>
       </c>
       <c r="Z23" t="n">
-        <v>1.626073835387846</v>
+        <v>1.146657787142027</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>inkling</t>
+          <t>k2-horizon-375b-a23b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Inkling (xhigh)</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Inkling</t>
+          <t>K2 Horizon 375B A23B</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Thinking Machines</t>
+          <t>MBZUAI Institute of Foundation Models</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>thinking-machines</t>
+          <t>mbzuai</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2571,82 +2571,54 @@
         <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>25.5423060999384</v>
+        <v>30.7949302696723</v>
       </c>
       <c r="K24" t="inlineStr"/>
-      <c r="L24" t="n">
-        <v>0.09468799999999999</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.002374</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0.001895</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0.09042</v>
-      </c>
-      <c r="P24" t="n">
-        <v>328.9</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>22793.6</v>
-      </c>
-      <c r="R24" t="n">
-        <v>467.8</v>
-      </c>
-      <c r="S24" t="n">
-        <v>22325.9</v>
-      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
-      <c r="U24" t="n">
-        <v>269.7523033535232</v>
-      </c>
-      <c r="V24" t="n">
-        <v>4.659587613245072</v>
-      </c>
-      <c r="W24" t="n">
-        <v>0.07765979355408453</v>
-      </c>
-      <c r="X24" t="n">
-        <v>0.003707104582864127</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>69.30252356339312</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>1.12059113522824</v>
-      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
+          <t>minimax-m3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Nemotron 3 Ultra</t>
+          <t>MiniMax-M3</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>MiniMax</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>nvidia</t>
+          <t>minimax</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2661,177 +2633,177 @@
         <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>23.4145123422858</v>
+        <v>29.6125932236316</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
-        <v>0.034269</v>
+        <v>0.026465</v>
       </c>
       <c r="M25" t="n">
-        <v>0.001525</v>
+        <v>0.004611</v>
       </c>
       <c r="N25" t="n">
-        <v>0.002978</v>
+        <v>0.00061</v>
       </c>
       <c r="O25" t="n">
-        <v>0.029765</v>
+        <v>0.021244</v>
       </c>
       <c r="P25" t="n">
-        <v>72.09999999999999</v>
+        <v>196.3</v>
       </c>
       <c r="Q25" t="n">
-        <v>12593.6</v>
+        <v>18211.1</v>
       </c>
       <c r="R25" t="n">
-        <v>1145.5</v>
+        <v>508</v>
       </c>
       <c r="S25" t="n">
-        <v>11448.1</v>
+        <v>17703.1</v>
       </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="n">
-        <v>683.2563641275146</v>
+        <v>1118.934185665279</v>
       </c>
       <c r="V25" t="n">
-        <v>19.48503107541121</v>
+        <v>9.051225641456423</v>
       </c>
       <c r="W25" t="n">
-        <v>0.3247505179235201</v>
+        <v>0.1508537606909404</v>
       </c>
       <c r="X25" t="n">
-        <v>0.00146357948861106</v>
+        <v>0.0008937076128435877</v>
       </c>
       <c r="Y25" t="n">
-        <v>174.6685159500694</v>
+        <v>92.77177789098317</v>
       </c>
       <c r="Z25" t="n">
-        <v>1.859239005708122</v>
+        <v>1.626073835387846</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>gemini-3-5-flash-lite</t>
+          <t>inkling</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Inkling (xhigh)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Gemini 3.5 Flash-Lite</t>
+          <t>Inkling</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Thinking Machines</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>thinking-machines</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H26" t="b">
         <v>1</v>
       </c>
       <c r="I26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>22.6606674839812</v>
+        <v>25.5423060999384</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
-        <v>0.019232</v>
+        <v>0.09468799999999999</v>
       </c>
       <c r="M26" t="n">
-        <v>0.000782</v>
+        <v>0.002374</v>
       </c>
       <c r="N26" t="n">
-        <v>0.001426</v>
+        <v>0.001895</v>
       </c>
       <c r="O26" t="n">
-        <v>0.017024</v>
+        <v>0.09042</v>
       </c>
       <c r="P26" t="n">
-        <v>20.3</v>
+        <v>254.3</v>
       </c>
       <c r="Q26" t="n">
-        <v>7379.9</v>
+        <v>22793.6</v>
       </c>
       <c r="R26" t="n">
-        <v>570.5</v>
+        <v>467.8</v>
       </c>
       <c r="S26" t="n">
-        <v>6809.5</v>
+        <v>22325.9</v>
       </c>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="n">
-        <v>1178.279299291868</v>
+        <v>269.7523033535232</v>
       </c>
       <c r="V26" t="n">
-        <v>66.97734231718582</v>
+        <v>6.026497703485269</v>
       </c>
       <c r="W26" t="n">
-        <v>1.116289038619763</v>
+        <v>0.1004416283914212</v>
       </c>
       <c r="X26" t="n">
-        <v>0.000848695212248054</v>
+        <v>0.003707104582864127</v>
       </c>
       <c r="Y26" t="n">
-        <v>363.5418719211822</v>
+        <v>89.63271726307509</v>
       </c>
       <c r="Z26" t="n">
-        <v>3.070592756538869</v>
+        <v>1.12059113522824</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>muse-glimmer</t>
+          <t>nvidia-nemotron-3-ultra-550b-a55b</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Nemotron 3 Ultra 550B A55B (Reasoning)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Muse Glimmer (high)</t>
+          <t>Nemotron 3 Ultra</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Meta</t>
+          <t>NVIDIA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>nvidia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>small</t>
+          <t>large</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -2841,82 +2813,82 @@
         <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>18.0678176089465</v>
+        <v>23.4145123422858</v>
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
-        <v>0.012326</v>
+        <v>0.034269</v>
       </c>
       <c r="M27" t="n">
-        <v>0.00072</v>
+        <v>0.001525</v>
       </c>
       <c r="N27" t="n">
-        <v>0.00067</v>
+        <v>0.002978</v>
       </c>
       <c r="O27" t="n">
-        <v>0.010936</v>
+        <v>0.029765</v>
       </c>
       <c r="P27" t="n">
-        <v>75.2</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="Q27" t="n">
-        <v>7737.1</v>
+        <v>12593.6</v>
       </c>
       <c r="R27" t="n">
-        <v>446.4</v>
+        <v>1145.5</v>
       </c>
       <c r="S27" t="n">
-        <v>7290.7</v>
+        <v>11448.1</v>
       </c>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="n">
-        <v>1465.829758960449</v>
+        <v>683.2563641275146</v>
       </c>
       <c r="V27" t="n">
-        <v>14.41581192203178</v>
+        <v>21.6466986215277</v>
       </c>
       <c r="W27" t="n">
-        <v>0.240263532033863</v>
+        <v>0.360778310358795</v>
       </c>
       <c r="X27" t="n">
-        <v>0.0006822074622834709</v>
+        <v>0.00146357948861106</v>
       </c>
       <c r="Y27" t="n">
-        <v>102.8869680851064</v>
+        <v>194.0462249614792</v>
       </c>
       <c r="Z27" t="n">
-        <v>2.335218312926871</v>
+        <v>1.859239005708122</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>mistral-medium-3-5</t>
+          <t>gemini-3-5-flash-lite</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mistral Medium 3.5</t>
+          <t>Gemini 3.5 Flash-Lite</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Mistral</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mistral</t>
+          <t>google</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2928,90 +2900,90 @@
         <v>1</v>
       </c>
       <c r="I28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>14.8946727802691</v>
+        <v>22.6606674839812</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
-        <v>0.108206</v>
+        <v>0.019232</v>
       </c>
       <c r="M28" t="n">
-        <v>0.002141</v>
+        <v>0.000782</v>
       </c>
       <c r="N28" t="n">
-        <v>0.058389</v>
+        <v>0.001426</v>
       </c>
       <c r="O28" t="n">
-        <v>0.047676</v>
+        <v>0.017024</v>
       </c>
       <c r="P28" t="n">
-        <v>84.5</v>
+        <v>19.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>14142</v>
+        <v>7379.9</v>
       </c>
       <c r="R28" t="n">
-        <v>7785.3</v>
+        <v>570.5</v>
       </c>
       <c r="S28" t="n">
-        <v>6356.8</v>
+        <v>6809.5</v>
       </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="n">
-        <v>137.6510801644003</v>
+        <v>1178.279299291868</v>
       </c>
       <c r="V28" t="n">
-        <v>10.57609901557569</v>
+        <v>68.32362055471718</v>
       </c>
       <c r="W28" t="n">
-        <v>0.1762683169262615</v>
+        <v>1.138727009245287</v>
       </c>
       <c r="X28" t="n">
-        <v>0.007264745026378824</v>
+        <v>0.000848695212248054</v>
       </c>
       <c r="Y28" t="n">
-        <v>167.3609467455621</v>
+        <v>370.8492462311558</v>
       </c>
       <c r="Z28" t="n">
-        <v>1.053222513100629</v>
+        <v>3.070592756538869</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>gpt-oss-120b</t>
+          <t>muse-glimmer</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>gpt-oss-120b (high)</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>gpt-oss-120b (high)</t>
+          <t>Muse Glimmer (high)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>openai</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2025-08-05</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>small</t>
         </is>
       </c>
       <c r="H29" t="b">
@@ -3021,50 +2993,230 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>12.3483931512592</v>
+        <v>18.0678176089465</v>
       </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
-        <v>0.007271</v>
+        <v>0.012326</v>
       </c>
       <c r="M29" t="n">
-        <v>0.000449</v>
+        <v>0.00072</v>
       </c>
       <c r="N29" t="n">
-        <v>0.000691</v>
+        <v>0.00067</v>
       </c>
       <c r="O29" t="n">
-        <v>0.006131</v>
+        <v>0.010936</v>
       </c>
       <c r="P29" t="n">
-        <v>50.9</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="Q29" t="n">
-        <v>11465.4</v>
+        <v>7737.1</v>
       </c>
       <c r="R29" t="n">
-        <v>1161.3</v>
+        <v>446.4</v>
       </c>
       <c r="S29" t="n">
-        <v>10304</v>
+        <v>7290.7</v>
       </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="n">
+        <v>1465.829758960449</v>
+      </c>
+      <c r="V29" t="n">
+        <v>12.62012871404878</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0.2103354785674796</v>
+      </c>
+      <c r="X29" t="n">
+        <v>0.0006822074622834709</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>90.0710128055879</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>2.335218312926871</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>mistral-medium-3-5</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Mistral Medium 3.5</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Mistral Medium 3.5</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Mistral</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>mistral</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H30" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>14.8946727802691</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>0.108206</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.002141</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.058389</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.047676</v>
+      </c>
+      <c r="P30" t="n">
+        <v>84.09999999999999</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>14142</v>
+      </c>
+      <c r="R30" t="n">
+        <v>7785.3</v>
+      </c>
+      <c r="S30" t="n">
+        <v>6356.8</v>
+      </c>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="n">
+        <v>137.6510801644003</v>
+      </c>
+      <c r="V30" t="n">
+        <v>10.62640150792088</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0.1771066917986814</v>
+      </c>
+      <c r="X30" t="n">
+        <v>0.007264745026378824</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>168.1569560047563</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>1.053222513100629</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b (high)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>gpt-oss-120b (high)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2025-08-05</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H31" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" t="b">
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>12.3483931512592</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="n">
+        <v>0.007271</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.000449</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.000691</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.006131</v>
+      </c>
+      <c r="P31" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>11465.4</v>
+      </c>
+      <c r="R31" t="n">
+        <v>1161.3</v>
+      </c>
+      <c r="S31" t="n">
+        <v>10304</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="n">
         <v>1698.307406307138</v>
       </c>
-      <c r="V29" t="n">
-        <v>14.55606265374366</v>
-      </c>
-      <c r="W29" t="n">
-        <v>0.2426010442290609</v>
-      </c>
-      <c r="X29" t="n">
+      <c r="V31" t="n">
+        <v>13.02115270783044</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0.217019211797174</v>
+      </c>
+      <c r="X31" t="n">
         <v>0.000588821550377877</v>
       </c>
-      <c r="Y29" t="n">
-        <v>225.2534381139489</v>
-      </c>
-      <c r="Z29" t="n">
+      <c r="Y31" t="n">
+        <v>201.5008787346221</v>
+      </c>
+      <c r="Z31" t="n">
         <v>1.077013724009559</v>
       </c>
     </row>

</xml_diff>